<commit_message>
05-08-2026 all data uploaded
</commit_message>
<xml_diff>
--- a/Data_Analytics/module-3-working-with-Python/advanced-python/file-handeling/workbook1.xlsx
+++ b/Data_Analytics/module-3-working-with-Python/advanced-python/file-handeling/workbook1.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7020" activeTab="2"/>
+    <workbookView windowWidth="20490" windowHeight="7620" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="employe_data" sheetId="1" r:id="rId1"/>
@@ -69,14 +69,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -538,148 +531,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>

</xml_diff>